<commit_message>
new rates simple and express
</commit_message>
<xml_diff>
--- a/calc/files/letter.xlsx
+++ b/calc/files/letter.xlsx
@@ -43,18 +43,19 @@
     <t>за каждые последующие полные или неполные 20 г массы бандероли</t>
   </si>
   <si>
-    <t>Постановление МАРТ 18.06.2025 № 43</t>
-  </si>
-  <si/>
+    <t>Постановление МАРТ 10.03.2026 № 19 в действии с 22.03.2026</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" mc:Ignorable="co co-ooxml w14 x14 w15">
   <numFmts>
+    <numFmt co:extendedFormatCode="General" formatCode="General" numFmtId="1002"/>
+    <numFmt co:extendedFormatCode="0.00" formatCode="0.00" numFmtId="1003"/>
     <numFmt co:extendedFormatCode="General" formatCode="General" numFmtId="1001"/>
     <numFmt co:extendedFormatCode="General" formatCode="General" numFmtId="1000"/>
-    <numFmt co:extendedFormatCode="0.00" formatCode="0.00" numFmtId="1002"/>
+    <numFmt co:extendedFormatCode="0.00" formatCode="0.00" numFmtId="1004"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -77,19 +78,19 @@
       <sz val="14"/>
     </font>
     <font>
-      <color theme="1" tint="0"/>
-      <sz val="14"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <name val="Roboto"/>
       <color rgb="333333" tint="0"/>
       <sz val="12"/>
     </font>
     <font>
+      <name val="Arial"/>
       <color theme="1" tint="0"/>
       <sz val="10"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000000" tint="0"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -105,7 +106,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -164,6 +165,20 @@
       <right style="thin">
         <color rgb="000000" tint="0"/>
       </right>
+      <top style="thin">
+        <color rgb="000000" tint="0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="000000" tint="0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000000" tint="0"/>
+      </left>
+      <right style="thin">
+        <color rgb="000000" tint="0"/>
+      </right>
       <bottom style="thin">
         <color rgb="000000" tint="0"/>
       </bottom>
@@ -182,7 +197,7 @@
       <alignment shrinkToFit="false" vertical="bottom" wrapText="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="true" borderId="0" fillId="0" fontId="1" numFmtId="1000" quotePrefix="false">
       <alignment shrinkToFit="false" vertical="bottom" wrapText="false"/>
     </xf>
@@ -201,27 +216,30 @@
     <xf applyAlignment="true" applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="1" fillId="2" fontId="3" numFmtId="1000" quotePrefix="false">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="true" applyBorder="true" applyFill="false" applyFont="true" applyNumberFormat="true" borderId="1" fillId="0" fontId="4" numFmtId="1000" quotePrefix="false">
+    <xf applyAlignment="true" applyBorder="true" applyFill="false" applyFont="true" applyNumberFormat="true" borderId="5" fillId="0" fontId="2" numFmtId="1002" quotePrefix="false">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf applyAlignment="true" applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="4" fillId="2" fontId="2" numFmtId="1000" quotePrefix="false">
       <alignment vertical="top" wrapText="true"/>
     </xf>
-    <xf applyAlignment="true" applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="1" fillId="2" fontId="5" numFmtId="1000" quotePrefix="false">
+    <xf applyAlignment="true" applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="1" fillId="2" fontId="4" numFmtId="1000" quotePrefix="false">
       <alignment vertical="top"/>
     </xf>
-    <xf applyBorder="true" applyFill="false" applyFont="true" applyNumberFormat="true" borderId="1" fillId="0" fontId="6" numFmtId="1000" quotePrefix="false"/>
-    <xf applyAlignment="true" applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="5" fillId="2" fontId="2" numFmtId="1000" quotePrefix="false">
+    <xf applyBorder="true" applyFill="false" applyFont="true" applyNumberFormat="true" borderId="5" fillId="0" fontId="5" numFmtId="1002" quotePrefix="false"/>
+    <xf applyAlignment="true" applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="6" fillId="2" fontId="2" numFmtId="1000" quotePrefix="false">
       <alignment vertical="top"/>
     </xf>
-    <xf applyAlignment="true" applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="1" fillId="2" fontId="2" numFmtId="1002" quotePrefix="false">
+    <xf applyAlignment="true" applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="1" fillId="2" fontId="2" numFmtId="1003" quotePrefix="false">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="true" borderId="0" fillId="0" fontId="1" numFmtId="1002" quotePrefix="false">
+    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="true" borderId="0" fillId="0" fontId="6" numFmtId="1004" quotePrefix="false">
       <alignment shrinkToFit="false" vertical="bottom" wrapText="false"/>
     </xf>
-    <xf applyAlignment="true" applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="6" fillId="2" fontId="2" numFmtId="1002" quotePrefix="false">
+    <xf applyAlignment="true" applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="7" fillId="2" fontId="2" numFmtId="1003" quotePrefix="false">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="true" borderId="0" fillId="0" fontId="6" numFmtId="1002" quotePrefix="false">
+      <alignment shrinkToFit="false" vertical="bottom" wrapText="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -453,6 +471,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s"/>
+      <c r="D1" s="0" t="n"/>
     </row>
     <row customHeight="true" ht="29.25" outlineLevel="0" r="2">
       <c r="A2" s="4" t="n"/>
@@ -462,6 +481,7 @@
       <c r="C2" s="6" t="s">
         <v>3</v>
       </c>
+      <c r="D2" s="0" t="n"/>
     </row>
     <row customHeight="true" ht="41.9999847412109" outlineLevel="0" r="3">
       <c r="A3" s="7" t="s">
@@ -469,20 +489,21 @@
       </c>
       <c r="B3" s="8" t="n"/>
       <c r="C3" s="9" t="n"/>
+      <c r="D3" s="0" t="n"/>
     </row>
     <row outlineLevel="0" r="4">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="11" t="n">
-        <v>0.86</v>
+        <v>1.04</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>0.72</v>
+        <v>0.87</v>
       </c>
       <c r="D4" s="12" t="n">
         <f aca="false" ca="false" dt2D="false" dtr="false" t="normal">C4*0.2</f>
-        <v>0.144</v>
+        <v>0.17400000000000002</v>
       </c>
     </row>
     <row outlineLevel="0" r="5">
@@ -490,10 +511,10 @@
         <v>6</v>
       </c>
       <c r="B5" s="13" t="n">
-        <v>0.86</v>
+        <v>1.04</v>
       </c>
       <c r="C5" s="13" t="n">
-        <v>0.72</v>
+        <v>0.87</v>
       </c>
       <c r="D5" s="12" t="n"/>
     </row>
@@ -502,43 +523,98 @@
         <v>7</v>
       </c>
       <c r="B6" s="13" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C6" s="13" t="n">
         <v>0.07</v>
       </c>
-      <c r="C6" s="13" t="n">
-        <v>0.06</v>
-      </c>
+      <c r="D6" s="0" t="n"/>
     </row>
     <row outlineLevel="0" r="7">
       <c r="A7" s="10" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="13" t="n">
-        <v>0.86</v>
+        <v>1.04</v>
       </c>
       <c r="C7" s="13" t="n">
-        <v>0.72</v>
-      </c>
+        <v>0.87</v>
+      </c>
+      <c r="D7" s="0" t="n"/>
     </row>
     <row outlineLevel="0" r="8">
       <c r="A8" s="10" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="13" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C8" s="13" t="n">
         <v>0.07</v>
       </c>
-      <c r="C8" s="13" t="n">
-        <v>0.06</v>
-      </c>
+      <c r="D8" s="0" t="n"/>
+    </row>
+    <row outlineLevel="0" r="9">
+      <c r="A9" s="0" t="n"/>
+      <c r="B9" s="0" t="n"/>
+      <c r="C9" s="0" t="n"/>
+      <c r="D9" s="0" t="n"/>
+    </row>
+    <row outlineLevel="0" r="10">
+      <c r="A10" s="0" t="n"/>
+      <c r="B10" s="0" t="n"/>
+      <c r="C10" s="0" t="n"/>
+      <c r="D10" s="0" t="n"/>
+    </row>
+    <row outlineLevel="0" r="11">
+      <c r="A11" s="0" t="n"/>
+      <c r="B11" s="0" t="n"/>
+      <c r="C11" s="0" t="n"/>
+      <c r="D11" s="0" t="n"/>
+    </row>
+    <row outlineLevel="0" r="12">
+      <c r="A12" s="0" t="n"/>
+      <c r="B12" s="0" t="n"/>
+      <c r="C12" s="0" t="n"/>
+      <c r="D12" s="0" t="n"/>
     </row>
     <row outlineLevel="0" r="13">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="14" t="s">
         <v>10</v>
       </c>
+      <c r="B13" s="0" t="n"/>
+      <c r="C13" s="0" t="n"/>
+      <c r="D13" s="0" t="n"/>
+    </row>
+    <row outlineLevel="0" r="14">
+      <c r="A14" s="0" t="n"/>
+      <c r="B14" s="0" t="n"/>
+      <c r="C14" s="0" t="n"/>
+      <c r="D14" s="0" t="n"/>
+    </row>
+    <row outlineLevel="0" r="15">
+      <c r="A15" s="0" t="n"/>
+      <c r="B15" s="0" t="n"/>
+      <c r="C15" s="0" t="n"/>
+      <c r="D15" s="0" t="n"/>
+    </row>
+    <row outlineLevel="0" r="16">
+      <c r="A16" s="0" t="n"/>
+      <c r="B16" s="0" t="n"/>
+      <c r="C16" s="0" t="n"/>
+      <c r="D16" s="0" t="n"/>
+    </row>
+    <row outlineLevel="0" r="17">
+      <c r="A17" s="0" t="n"/>
+      <c r="B17" s="0" t="n"/>
+      <c r="C17" s="0" t="n"/>
+      <c r="D17" s="0" t="n"/>
     </row>
     <row outlineLevel="0" r="18">
-      <c r="B18" s="0" t="s">
-        <v>11</v>
-      </c>
+      <c r="A18" s="0" t="n"/>
+      <c r="B18" s="14" t="n"/>
+      <c r="C18" s="0" t="n"/>
+      <c r="D18" s="0" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>